<commit_message>
Archive experimental artifacts and keep a production-grade locked layout.
Move chunks, chunk embeds, retrieve experiments, gold-4 report packs, and scratch reports into _archive; ship skill-named client roll-up and point retrieve/docs at the cleaned output surface.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/veramynd/veramynd_parser/output/reports/GA_ELA_G1_Module2_client_correlation.xlsx
+++ b/veramynd/veramynd_parser/output/reports/GA_ELA_G1_Module2_client_correlation.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_correlation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provenance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parent_rollup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provenance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -482,7 +483,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -494,7 +495,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -517,7 +518,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -529,7 +530,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -552,7 +553,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -564,7 +565,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -587,7 +588,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -599,7 +600,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -622,7 +623,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -634,7 +635,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -657,7 +658,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -669,7 +670,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -692,7 +693,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -704,7 +705,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -727,7 +728,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -739,7 +740,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -762,7 +763,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -774,7 +775,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -797,7 +798,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -809,7 +810,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -832,7 +833,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -844,7 +845,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -867,7 +868,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -879,7 +880,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -902,7 +903,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -914,7 +915,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -937,7 +938,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -949,7 +950,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -972,7 +973,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -984,7 +985,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1007,7 +1008,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1019,7 +1020,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1042,7 +1043,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1054,7 +1055,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1077,7 +1078,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1089,7 +1090,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1112,7 +1113,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1124,7 +1125,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1147,7 +1148,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1159,7 +1160,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1182,7 +1183,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1194,7 +1195,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1217,7 +1218,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1229,7 +1230,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1252,7 +1253,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1264,7 +1265,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1287,7 +1288,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1299,7 +1300,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1357,7 +1358,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1369,7 +1370,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1392,7 +1393,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1404,7 +1405,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1462,8 +1463,8 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>This standard is partially met. The select clause is not met: students never choose their own texts — the teacher assigns the read-aloud ("Elvin, the Boy Who Loved the Sky") and the mystery sky photos.
-Module 2: pp. 48, 102</t>
+          <t>This standard is partially met. However, the select clause is not met — the teacher assigns the text and photos; students never choose their own texts. Per F13, write-without-select is partial, not none.
+Module 2: pp. 44, 99</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1533,27 +1534,23 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>This standard is partially met. The lesson partially meets 1.P.EICC.1.e. Students also review existing Classroom Discussion Norms ("Direct students' attention to the Classroom Discussion Norms anchor chart and quickly review their jobs as speakers and listeners"), which partially meets the develop-group-norms…
-Module 2: pp. 45, 58, 70, 79, 90, 109, 133, 145, 151, 163, 166, 180, 190, 205, 291, 313, 444</t>
+          <t>This standard is partially met. Students also review group norms via the Classroom Discussion Norms anchor chart, partially meeting the develop-norms clause.
+Module 2: pp. 45, 58, 70, 79, 90, 109, 133, 145, 151, 163, 180, 190, 291, 313, 444</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L7, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8, G1M2U3L11</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L7, G1M2U1L9, G1M2U2L10, G1M2U2L8, G1M2U3L11</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L13, G1M2U2L1</t>
-        </is>
-      </c>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1609,19 +1606,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>This standard is partially met. The interpretation (I) clause is only partially met: students interpret the model poem by identifying high-quality writing features ("What is something you saw or heard in the poem that let you know the poem is high quality?"), but this interpretation focuses on craft quality…
-Module 2: pp. 389</t>
+          <t>This standard is partially met. However, students do not construct/create their own story sharing a real or imagined experience in this lesson — the response sheet records details from the read-aloud text, not an original narrative.
+Module 2: pp. 70, 390</t>
         </is>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>G1M2U3L5</t>
+          <t>G1M2U1L3, G1M2U3L5</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -1645,26 +1642,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 59, 70, 79, 83, 102, 109, 118, 125, 141, 151, 161, 171, 180, 188, 205, 227, 237, 257, 279, 291, 301, 307, 324, 332, 350, 361, 366, 380, 399, 404, 414, 424, 445, 456, 463</t>
+          <t>Module 2: pp. 44, 59, 68, 79, 102, 109, 118, 141, 151, 161, 171, 188, 227, 237, 257, 279, 291, 301, 324, 332, 350, 361, 399, 445, 456, 463</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>26</v>
       </c>
       <c r="F35" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L6</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L5, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U3L3, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1684,26 +1677,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Module 2: pp. 43, 59, 70, 78, 89, 99, 109, 125, 141, 151, 161, 171, 180, 188, 213, 291, 311</t>
+          <t>Module 2: pp. 44, 59, 70, 78, 89, 103, 109, 141, 161, 171, 180, 188, 213, 291, 311</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L9</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1723,22 +1712,21 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>This standard is partially met. partial-or-none — The interpretation clause is partially met: students are asked "What is something you saw or heard in the poem that let you know the poem is high quality?" which invites evaluative noticing of the model poem, but the act stays at the observational/noticing…
-Module 2: pp. 389</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>G1M2U3L5</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1759,7 +1747,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1771,7 +1759,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -1794,7 +1782,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1806,7 +1794,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -1829,7 +1817,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1841,7 +1829,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -1864,7 +1852,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1876,7 +1864,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -1899,7 +1887,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1911,7 +1899,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -1934,8 +1922,8 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>This standard is partially met. The make-predictions clause is partially met: in Opening A, students are asked "Based on the title of the story, what do you think this story will be about?" and they respond with predictions (e.g., "a little boy who likes things in the sky").
-Module 2: pp. 43, 99</t>
+          <t>This standard is partially met. However, there is no activity where students track or revisit their predictions as the reading progresses — the lesson moves through paragraphs with comprehension questions but never returns to confirm or revise the initial prediction.
+Module 2: pp. 44, 99</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1949,16 +1937,8 @@
           <t>G1M2U1L1, G1M2U1L6</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>input_scope_caveat present on one or more lesson rows</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1978,8 +1958,8 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>This standard is partially met. partial-or-full — The make clause is partially met: students are directed to infer why the sun will be at one corner of the page ("With your partner, discuss why you think the sun will be at one corner of the page at the end of the story.
-Module 2: pp. 99</t>
+          <t>This standard is partially met. partial-or-none — In the Mini Language Dive (For ELLs), students infer the meaning of a verse: "What does this verse mean?" (Responses will vary.) and "Now what do you think the verse means?" — a genuine make-inference act about meaning within the text.
+Module 2: pp. 100</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1993,16 +1973,8 @@
           <t>G1M2U1L6</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>input_scope_caveat present on one or more lesson rows</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2022,7 +1994,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Module 2: pp. 99, 151, 161</t>
+          <t>Module 2: pp. 100, 151, 161</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2057,7 +2029,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2069,7 +2041,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2092,7 +2064,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2104,7 +2076,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2127,18 +2099,18 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Module 2: pp. 58, 91, 99, 134, 144, 188, 213, 289, 311</t>
+          <t>Module 2: pp. 44, 58, 66, 91, 100, 134, 144, 188, 213, 289, 311</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2162,26 +2134,22 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Module 2: pp. 125, 290, 312, 323, 381, 409, 420, 428, 436</t>
+          <t>Module 2: pp. 290, 312, 323, 381, 409, 420, 428, 436</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>5</v>
       </c>
       <c r="F49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L8, G1M2U3L10, G1M2U3L4, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U2L10, G1M2U2L11, G1M2U2L8, G1M2U3L10, G1M2U3L4, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L9</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2236,26 +2204,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Module 2: pp. 375, 391, 423, 430, 432, 447</t>
+          <t>Module 2: pp. 392, 423, 430, 447</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U3L11, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10, G1M2U3L4</t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2311,7 +2275,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2323,7 +2287,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2346,19 +2310,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>This standard is partially met. The lesson partially addresses 1.P.ST.1.a. However, these discussions focus on noticing and wondering about content rather than explicitly identifying the key components of context most relevant to interpreting or constructing texts.
-Module 2: pp. 43, 99</t>
+          <t>This standard is partially met. However, per F21, the research clause is not met — the teacher-assigned read-aloud, photos, and videos are content delivery, not student-initiated informal research.
+Module 2: pp. 47</t>
         </is>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L6</t>
+          <t>G1M2U1L1</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -2382,7 +2346,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2394,7 +2358,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2488,7 +2452,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2500,7 +2464,7 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -2559,7 +2523,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the lesson does not have students analyze how these elements affect the audience or explain/evaluate how they support the text's purpose; those higher-order clauses are entirely absent.
+          <t>This standard is partially met. However, no activity asks students to analyze or explain how these elements affect the audience or support the text's purpose — the analyze/explain clause is not met.
 Module 2: pp. 70</t>
         </is>
       </c>
@@ -2595,7 +2559,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2607,7 +2571,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -2630,7 +2594,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2642,7 +2606,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -2665,7 +2629,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2677,7 +2641,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -2700,7 +2664,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2712,7 +2676,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -2735,27 +2699,23 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>This standard is partially met. [REJECTED: evidence missing or not found in lesson raw text].
-Module 2: pp. 381, 389, 432</t>
+          <t>This standard is partially met. Students craft words and phrases for their poem verse using the Adjectives anchor chart and model poem (Work Time A-B), and write a closing to "tell the reader that night is coming to an end." However, the lesson does not explicitly direct students to consider how their…
+Module 2: pp. 390</t>
         </is>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>G1M2U3L10, G1M2U3L4, G1M2U3L5</t>
+          <t>G1M2U3L5</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10</t>
-        </is>
-      </c>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2775,7 +2735,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2787,7 +2747,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -2810,7 +2770,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2822,7 +2782,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -2845,26 +2805,23 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Module 2: pp. 217, 389, 432</t>
+          <t>This standard is partially met. The explore/interpret side is thin: students answer one question about high-quality features in the model poem (Opening A: "What is something you saw or heard in the poem that let you know the poem is high quality?") but do not substantively analyze how features impact meaning,…
+Module 2: pp. 389</t>
         </is>
       </c>
       <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
         <v>1</v>
       </c>
-      <c r="F68" t="n">
-        <v>2</v>
-      </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>G1M2U2L2, G1M2U3L10, G1M2U3L5</t>
+          <t>G1M2U3L5</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L2, G1M2U3L10</t>
-        </is>
-      </c>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2884,7 +2841,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -2896,7 +2853,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -2919,7 +2876,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2931,7 +2888,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -2954,26 +2911,23 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Module 2: pp. 235, 281, 364, 375, 389, 394, 418, 432</t>
+          <t>This standard is partially met. The consume clause is partially met: students engage with multiple modes — a poem ("Display the 'What We See: The Sun, Moon, and Stars' poem"), photographs ("Display sun photograph 2 and moon photograph 2"), and a video ("As they watch the video, they should look carefully to…
+Module 2: pp. 235, 281, 364, 418</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>G1M2U2L3, G1M2U2L7, G1M2U3L10, G1M2U3L2, G1M2U3L4, G1M2U3L5, G1M2U3L6, G1M2U3L8</t>
+          <t>G1M2U2L3, G1M2U2L7, G1M2U3L2, G1M2U3L8</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10, G1M2U3L4, G1M2U3L6</t>
-        </is>
-      </c>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2993,7 +2947,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -3005,7 +2959,7 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3063,18 +3017,18 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 171, 381, 389, 419, 428, 436, 444</t>
+          <t>Module 2: pp. 45, 171, 381, 389, 419, 428, 444</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" t="n">
         <v>3</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L13, G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L13, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -3098,18 +3052,18 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Module 2: pp. 47, 58, 81, 89, 99, 109, 118, 130, 145, 151, 161, 188, 214, 223, 235, 245, 255, 268, 279, 301, 313, 324, 332, 352, 365, 373, 381, 399, 408, 419, 428, 436, 448, 456, 463</t>
+          <t>Module 2: pp. 45, 58, 70, 81, 89, 99, 109, 118, 130, 145, 151, 161, 188, 214, 223, 235, 245, 255, 268, 279, 301, 313, 324, 332, 352, 365, 373, 381, 389, 399, 408, 419, 428, 436, 448, 456, 463</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L15, G1M2U1L2, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -3133,26 +3087,22 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 51, 70, 81, 92, 99, 109, 117, 125, 141, 146, 161, 171, 180, 188, 205, 223, 246, 259, 268, 291, 301, 313, 332, 352, 364, 373, 379, 389, 408, 421, 430, 438, 448, 457, 463</t>
+          <t>Module 2: pp. 45, 70, 81, 92, 103, 109, 117, 141, 161, 171, 180, 188, 223, 246, 259, 268, 291, 301, 313, 332, 352, 364, 373, 379, 389, 408, 421, 430, 438, 448, 457, 463</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L12, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L10, G1M2U2L12, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L11, G1M2U1L2, G1M2U1L9, G1M2U2L1</t>
-        </is>
-      </c>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3172,7 +3122,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -3184,7 +3134,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3207,7 +3157,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -3219,7 +3169,7 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3242,8 +3192,8 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>This standard is partially met. The ask clause is not fully met: students are prompted to share "wonders" using the frame "I wonder ___________," and the ELL scaffold models wonder-to-question conversion, but the lesson never scripts a moment where students pose a genuine question to a partner or audience…
-Module 2: pp. 47, 61, 99</t>
+          <t>This standard is partially met. However, the ask clause is not met — every text-dependent and discussion question is teacher-posed; students only respond.
+Module 2: pp. 47, 70, 102</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -3257,16 +3207,8 @@
           <t>G1M2U1L1, G1M2U1L3, G1M2U1L6</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>input_scope_caveat present on one or more lesson rows; missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L3</t>
-        </is>
-      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3321,7 +3263,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -3333,7 +3275,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -3356,7 +3298,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -3368,7 +3310,7 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -3391,7 +3333,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -3403,7 +3345,7 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -3426,7 +3368,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -3438,7 +3380,7 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -3461,7 +3403,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3473,7 +3415,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -3496,7 +3438,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -3508,7 +3450,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -3531,7 +3473,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -3543,7 +3485,7 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -3566,7 +3508,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -3578,7 +3520,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -3601,7 +3543,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3613,7 +3555,7 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -3636,7 +3578,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3648,7 +3590,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -3671,7 +3613,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -3683,7 +3625,7 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -3706,7 +3648,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -3718,7 +3660,7 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -3741,7 +3683,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3753,7 +3695,7 @@
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -3776,7 +3718,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -3788,7 +3730,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -3811,7 +3753,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -3823,7 +3765,7 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -3846,7 +3788,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -3858,7 +3800,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -3881,7 +3823,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -3893,7 +3835,7 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -3916,7 +3858,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -3928,7 +3870,7 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -3951,7 +3893,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the lesson never explicitly addresses using a VARIETY of simple sentences or varying sentence TYPES (declarative, interrogative, exclamatory, imperative) — the writing task is structured around a poem model and verse planner, producing sentences but not deliberately…
+          <t>This standard is partially met. Students independently write verse 3 in complete sentences (Work Time B, p.390): the teacher feedback confirms students turn ideas "into a complete sentence." However, the lesson does not explicitly direct students to use a variety of sentence types or focus on sentence variety…
 Module 2: pp. 390</t>
         </is>
       </c>
@@ -3987,7 +3929,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -3999,7 +3941,7 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -4022,7 +3964,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -4034,7 +3976,7 @@
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -4057,7 +3999,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 70, 99, 389</t>
+          <t>Module 2: pp. 46, 68, 100, 390</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -4092,8 +4034,8 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the vocabulary deployment is thin: students use basic content-label words within heavily scaffolded sentence frames rather than demonstrating robust, self-generated use of grade-level vocabulary to communicate meaning.
-Module 2: pp. 39, 99, 389</t>
+          <t>This standard is partially met. However, the deployment occurs primarily in oral partner/small-group discussion settings; the response sheet writing is not explicitly shown to require target vocabulary deployment.
+Module 2: pp. 48, 103, 389</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -4108,11 +4050,7 @@
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L1</t>
-        </is>
-      </c>
+      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4132,7 +4070,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -4144,7 +4082,7 @@
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -4167,7 +4105,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -4179,7 +4117,7 @@
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -4202,14 +4140,15 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Module 2: pp. 99</t>
+          <t>This standard is partially met. However, per R3, this act occurs only in supplemental (For ELLs) content, capping the clause at partial.
+Module 2: pp. 100</t>
         </is>
       </c>
       <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
         <v>1</v>
-      </c>
-      <c r="F106" t="n">
-        <v>0</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -4237,7 +4176,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -4249,7 +4188,7 @@
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -4272,7 +4211,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -4284,7 +4223,7 @@
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -4307,7 +4246,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -4319,7 +4258,7 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -4342,7 +4281,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Module 2: pp. 99, 389</t>
+          <t>Module 2: pp. 100, 390</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -4413,7 +4352,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4425,7 +4364,7 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -4448,26 +4387,22 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Module 2: pp. 59, 91, 109, 121, 134, 144, 154, 164, 173, 180, 188, 249, 257, 262, 283, 290, 295, 312, 325, 332, 381, 390, 420, 429, 438, 447, 467</t>
+          <t>Module 2: pp. 59, 91, 109, 121, 134, 144, 154, 164, 173, 180, 188, 249, 257, 283, 290, 312, 325, 332, 381, 390, 420, 429, 438, 447, 467</t>
         </is>
       </c>
       <c r="E113" t="n">
         <v>24</v>
       </c>
       <c r="F113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L10, G1M2U3L11, G1M2U3L13, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L4, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U3L10, G1M2U3L11, G1M2U3L13, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U2L9</t>
-        </is>
-      </c>
+      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4487,7 +4422,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4499,7 +4434,7 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -4522,7 +4457,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4534,7 +4469,7 @@
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -4557,7 +4492,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4569,7 +4504,7 @@
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -4592,27 +4527,23 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, within this lesson the student uses only one pre-supplied transition phrase ("At the end") in a scaffolded frame rather than independently selecting and deploying multiple transition words/phrases (e.g., once upon a time, next, last) to sequence events and actions.
-Module 2: pp. 94, 125</t>
+          <t>This standard is partially met. Per F14, a scaffolded (C) frame in which the student performs the act floors at partial, never none. However, the transition phrase is pre-printed (not student-selected) and is a single use, so the standard is only partially met.
+Module 2: pp. 102</t>
         </is>
       </c>
       <c r="E117" t="n">
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>G1M2U1L6, G1M2U1L9</t>
+          <t>G1M2U1L6</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L6, G1M2U1L9</t>
-        </is>
-      </c>
+      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4632,26 +4563,22 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Module 2: pp. 66, 121, 141, 180, 233, 244, 262, 279, 380, 399, 404, 444</t>
+          <t>Module 2: pp. 67, 121, 141, 180, 233, 244, 279, 380, 399, 444</t>
         </is>
       </c>
       <c r="E118" t="n">
         <v>5</v>
       </c>
       <c r="F118" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L14, G1M2U1L3, G1M2U1L8, G1M2U2L3, G1M2U2L4, G1M2U2L6, G1M2U2L7, G1M2U3L11, G1M2U3L4, G1M2U3L6, G1M2U3L7</t>
+          <t>G1M2U1L10, G1M2U1L14, G1M2U1L3, G1M2U1L8, G1M2U2L3, G1M2U2L4, G1M2U2L7, G1M2U3L11, G1M2U3L4, G1M2U3L6</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U3L7</t>
-        </is>
-      </c>
+      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4671,26 +4598,22 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Module 2: pp. 121, 144, 180, 222, 249, 260, 262, 283, 293, 295, 316, 325, 381, 389, 420, 428, 432, 445</t>
+          <t>Module 2: pp. 121, 144, 180, 222, 249, 260, 283, 293, 316, 325, 381, 390, 420, 428, 445</t>
         </is>
       </c>
       <c r="E119" t="n">
         <v>6</v>
       </c>
       <c r="F119" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L14, G1M2U1L8, G1M2U2L10, G1M2U2L11, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L10, G1M2U1L14, G1M2U1L8, G1M2U2L10, G1M2U2L11, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U2L9, G1M2U3L10</t>
-        </is>
-      </c>
+      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4711,7 +4634,7 @@
       <c r="D120" t="inlineStr">
         <is>
           <t>This standard is partially met. The major events clause is only partially met — students discuss what Moon saw and why he changed his mind, but the lesson explicitly defers completing the events section of the Story Elements board to the next lesson, and no question directly asks students to identify the…
-Module 2: pp. 70, 99, 109, 141, 161, 171, 180</t>
+Module 2: pp. 70, 100, 109, 141, 161, 171, 180</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4790,18 +4713,18 @@
       <c r="D122" t="inlineStr">
         <is>
           <t>This standard is partially met. (bored and lonely)") and on the response sheet using a word bank of adjectives (curious, bored, angry, confused) with the frame "I think Moon was _________ because __________." The clause "explain how the characters' actions support the central message, lesson, or moral" is…
-Module 2: pp. 118, 141, 151, 180</t>
+Module 2: pp. 100, 118, 141, 151, 180</t>
         </is>
       </c>
       <c r="E122" t="n">
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L14, G1M2U1L8</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L14, G1M2U1L6, G1M2U1L8</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -4825,7 +4748,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4837,7 +4760,7 @@
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -4860,7 +4783,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4872,7 +4795,7 @@
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -4931,7 +4854,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4943,7 +4866,7 @@
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -4966,7 +4889,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4978,7 +4901,7 @@
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
@@ -5001,7 +4924,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -5013,7 +4936,7 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -5036,7 +4959,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -5048,7 +4971,7 @@
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -5071,7 +4994,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -5083,7 +5006,7 @@
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -5106,26 +5029,22 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Module 2: pp. 380, 390, 419, 429, 432, 445</t>
+          <t>Module 2: pp. 390, 419, 429, 445</t>
         </is>
       </c>
       <c r="E131" t="n">
         <v>4</v>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U3L11, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10</t>
-        </is>
-      </c>
+      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5145,7 +5064,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45</t>
+          <t>Module 2: pp. 48</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -5215,26 +5134,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 59, 70, 79, 91, 102, 109, 121, 125, 141, 146, 161, 180, 190, 215, 222, 233, 248, 259, 268, 279, 291, 306, 313, 324, 332, 352, 361, 373, 381, 399, 408, 419, 429, 438, 448, 455, 463</t>
+          <t>Module 2: pp. 49, 59, 70, 79, 91, 103, 109, 121, 141, 161, 180, 190, 215, 222, 233, 248, 259, 268, 279, 291, 306, 313, 324, 332, 352, 361, 373, 381, 399, 408, 419, 429, 438, 448, 455, 463</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F134" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L11, G1M2U1L9</t>
-        </is>
-      </c>
+      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5254,18 +5169,18 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Module 2: pp. 51, 91, 94, 130, 141, 151, 161, 171, 180, 188, 213, 312</t>
+          <t>Module 2: pp. 91, 100, 130, 141, 151, 161, 171, 180, 188, 213, 312</t>
         </is>
       </c>
       <c r="E135" t="n">
         <v>5</v>
       </c>
       <c r="F135" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -5275,7 +5190,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>input_scope_caveat present on one or more lesson rows; missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L2, G1M2U1L6</t>
+          <t>input_scope_caveat present on one or more lesson rows</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5212,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -5309,7 +5224,7 @@
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of Module 2.</t>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -5325,87 +5240,916 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>field</t>
+          <t>Standard Section</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>Parent Standard</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Alignment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Roll-up statement — CLIENT FORMAT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>client_format_version</t>
+          <t>Foundations</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.1-client-ga-ela</t>
+          <t>1.F.F.1 — Oral &amp; Silent Reading Fluency: Demonstrate oral and silent reading fluency while reading grade-level texts for understanding, self-correcting as necessary to ensure accuracy and aid comprehension.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>program_name</t>
+          <t>Foundations</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EL Education Curriculum</t>
+          <t>1.F.H.1 — Motor Skills &amp; Letter/Word Formation: Use fine motor skills to form legible letters and words in print.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>Foundations</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Veramynd_ALL40_corrected_master.xlsx</t>
+          <t>1.F.H.2 — Transcription &amp; Handwriting Fluency: Use working memory to transcribe oral language to written text and maintain meaning while writing letters, words, and sentences quickly and accurately.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support perform basic transcription skills. However, the citations do not cover the standard's other intended skills: build handwriting fluency by forming accurate letters and words with increasing speed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>include_statuses</t>
+          <t>Foundations</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>full,partial</t>
+          <t>1.F.P.1 — Phoneme-Grapheme Correspondences: Identify and produce phoneme-grapheme correspondences.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>leaf_standards_with_citations</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>51</v>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.F.P.2 — Decoding with Phonics: Use grade-level phonics skills to decode words in context and in isolation.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1.F.P.3 — Encoding with Phonics: Use grade-level phonics skills to encode words in context and in isolation.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1.F.PA.4 — Syllables: Identify and manipulate syllables in spoken words.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1.F.PA.5 — Onsets &amp; Rimes: Blend and segment onsets and rimes in spoken words.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1.F.PA.6 — Phonemic Awareness: Identify and manipulate the individual sounds in spoken words.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1.L.GC.1 — Grammar, Usage, &amp; Mechanics: Learn and apply conventions of Standard English grammar, usage, and mechanics to aid the comprehension of texts and to communicate clearly in written and spoken language.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1.L.GC.2 — Syntax: Recognize and compose coherent sentences that express complete thoughts.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support use a variety of simple sentences (including a variety of sentence types) to develop clarity in written texts. However, the citations do not cover the standard's other intended skills: distinguish between complete and incomplete simple sentences, and identify the sentence type (i.e., declarative, imperative, interrogative, and exclamatory), use singular and plural subjects with matching verbs, and with adult support, use adjectives or adverbs to add details or clarify meaning. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1.L.V.1 — General, Academic, &amp; Specialized Vocabulary: Acquire and use general, academic, and specialized vocabulary words and phrases in a variety of settings.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support acquire and apply general, academic, and specialized vocabulary words and phrases through grade-level texts and content and use grade-level general, academic, and specialized vocabulary words and phrases to communicate in a variety of settings. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1.L.V.2 — Word Analysis: Acquire and apply word analysis skills to deconstruct and construct words to make meaning.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1.L.V.3 — Meaning &amp; Purpose: Make connections between words and phrases and use reference materials to determine or clarify word meanings in a variety of settings and for a variety of purposes.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support use knowledge of word relationships and learned vocabulary words and phrases when making word choices in speaking and writing and use context within and beyond a sentence to determine or clarify the meaning of unknown and multiple-meaning words and phrases. However, the citations do not cover the standard's other intended skills: identify the relationship between words and their synonyms and antonyms, distinguish shades of meaning among verbs that describe the same general action (e.g., walk, march, strut, prance), and with teacher support, use a picture dictionary or digital resource to clarify the meaning of unknown words and phrases. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1.P.AC.1 — Reading like a Writer: Interpret texts through the author’s lens by identifying, analyzing, and evaluating craft techniques that are connected to the responses, thoughts, decisions, and questions triggered by the text.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support identify, apply, and analyze the literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements in texts, explaining or evaluating how specific elements affect the target audience and support the text’s purpose. However, the citations do not cover the standard's other intended skills: identify, apply, and analyze important, interesting, or effective uses of language, explaining or evaluating how specific word choices affect the target audience and support the text’s purpose, explain, analyze, and evaluate how the author’s use of sentence structure and syntax affects the target audience and supports the text’s purpose, and describe, analyze, and evaluate the design and organization of the text, explaining how specific formats, structures, patterns, and features influence the audience, contribute to the text’s accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1.P.AC.2 — Writing like a Reader: Construct texts with the audience’s experience in mind, basing decisions about craft techniques on context and purpose.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support craft words and phrases in order to influence the responses, thoughts, decisions, and questions of the target audience and achieve a specific purpose. However, the citations do not cover the standard's other intended skills: integrate literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements to appeal to target audiences and achieve specific purposes, make decisions about sentence structure and syntax in order to accommodate and influence the audience and achieve a specific purpose, and organize texts by incorporating specific formats, structures, patterns, and features to influence the audience, facilitate accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1.P.AC.3 — Text Design: Consider the impact of text design on audience and purpose when consuming and producing texts across modes and genres.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support explore and create texts in various modes and genres, developing and applying knowledge of how specific features impact meaning, tone, style, purpose, and audience and consume and produce multimodal texts, integrating a variety of genres, text features, and craft techniques to influence target audiences and achieve specific purposes. However, the citations do not cover the standard's other intended skills: apply knowledge of how mode and genre impact what kinds of ideas and information are included in texts and apply knowledge of how mode and genre impact how ideas and information are structured and arranged in texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1.P.CP.1 — Collaboration: Collaborate with others to accomplish shared goals and projects.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support collaborate with others to determine group norms, establish goals and procedures, and facilitate productivity when working on shared projects, contribute to discussions and shared projects by offering ideas, listening to the ideas of others, and providing feedback, and work with others to discuss topics, investigate questions, solve problems, and explore and create texts. However, the citations do not cover the standard's other intended skills: arrive to group discussions and collaborative meetings prepared to be an active participant in the work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1.P.CP.2 — Presentation: Use presentation skills to tailor communication to target audiences for specific purposes.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support communicate clearly to present ideas, information, and texts, build background knowledge by reciting all or part of significant poems and speeches as appropriate by grade level, and engage in dialogue with audiences by asking and answering questions. However, the citations do not cover the standard's other intended skills: integrate modes and genres most appropriate to purpose and audience and vary tone, pace, and nonverbal gestures as appropriate to purpose and audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1.P.EICC.1 — Reader &amp; Writer Identity: Build an identity as a reader and writer, developing a repertoire of resources and tools to continuously expand participation as an active consumer and producer of texts.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support discuss or write about personal and academic reading and writing preferences, referring to specific techniques, topics, modes, and genres that resonate most, build a repertoire of comprehension and composition skills, strategies, and techniques, drawing from them as needed to aid the interpretation and construction of texts, select, read, and write texts of personal interest and academic relevance to grade-level texts and topics, participate in a community of readers and writers by developing group norms, discussing texts, sharing individual writing, listening as others share their writing, and offering and responding to feedback, and develop independence and autonomy as a reader and writer. However, the citations do not cover the standard's other intended skills: generate, understand, monitor, and discuss personal and academic reading and writing goals, revising as appropriate. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1.P.EICC.2 — Engagement &amp; Intention: Engage in written or spoken dialogue as author and audience for a variety of tasks and purposes, making intentional connections within, between, and beyond texts.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support make use of texts to build knowledge, develop skills, make informed decisions, and share information and ideas, explain and learn concepts and processes by interpreting and constructing texts, and share real or imagined experiences by interpreting and constructing texts that tell or include stories. However, the citations do not cover the standard's other intended skills: interpret and construct texts to aid the analysis and evaluation of texts and ideas and consume and produce texts in order to solve problems or influence decisions. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1.P.EICC.3 — Comprehension Strategies: Engage with a range of complex texts for a variety of tasks and purposes, accessing and using strategies for comprehension before, during, and after reading as part of the meaning-making process.
+Comprehension strategies are tools that students should develop throughout their K-12 education as they work to interpret increasingly complex texts. The effectiveness of these strategies depends largely on the texts themselves, the reasons students engage with them, and the preferences and knowledge bases of individual students. For these reasons, students should receive instruction in a variety of comprehension strategies. Students should learn to select and apply strategies flexibly in order to make sense of the text and accomplish their goals.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support determine the meanings of unfamiliar words and concepts by applying knowledge of context and of academic vocabulary and word parts, make and track predictions about the events and information likely to come next, and make, track, and support inferences about different levels of meaning within the text. However, the citations do not cover the standard's other intended skills: establish a purpose and set goals for reading, monitor comprehension, and adjust as needed, scan and skim the text, making note of structures and sections that might be most useful, draw from, compare, build, and integrate prior knowledge with the material in the text, addressing inconsistencies or gaps and adding to knowledge repertoires as appropriate, and summarize and visualize sections of the text to maintain understanding. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1.P.EICC.4 — Writing Processes: Compose a range of texts for a variety of purposes and audiences, flexibly engaging in writing processes to plan, draft, evaluate, revise, and edit texts.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support generate ideas for content by assessing prior knowledge, gathering information from texts, and engaging in discussions with others, link ideas and information to the organization plan, highlighting ideas and information that are most relevant, useful, and impactful, construct an initial draft by integrating ideas and information, evaluate the text’s effectiveness based on self-review or feedback from others, determining whether the text matches the purpose and goals for writing, and make changes to the text based on self-evaluation or external feedback, revising the organization, ideas, information, word choices, and craft techniques in order to increase the text’s effectiveness. However, the citations do not cover the standard's other intended skills: establish a purpose and goals for writing and identify a target audience, plan how to organize the text by selecting modes, genres, and structures that will achieve the purpose and meet the needs of the target audience, and edit the text, ensuring it adheres to the conventions of written language. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1.P.ST.1 — Context: Develop and apply knowledge of key components of context such as background information, geographic location, cultural influences, time period, and contemporary events when interpreting and constructing texts.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support use prior knowledge, formal or informal research, and discussions with others to identify the key components of context that are most relevant and explore how context shapes the author’s decisions and the audience’s responses during the interpretation and construction of texts. However, the citations do not cover the standard's other intended skills: consider how context impacts the purposes of the author and the audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Practices</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1.P.ST.2 — Author, Audience, &amp; Purpose: Interpret and construct texts by developing and applying knowledge of the strategies and techniques authors use to accommodate the target audience and achieve the text’s purpose.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support develop and apply knowledge of author, audience, and context to discern and establish the purpose of texts being interpreted or constructed and to evaluate the extent to which those texts achieve those purposes and draw from knowledge of how authors consider context and audience to determine which information and ideas to highlight, which text design is most accessible, which word choices and language structures are most effective, and which craft techniques are most impactful. However, the citations do not cover the standard's other intended skills: draw from knowledge of author, audience, and context to discern and establish a clear point of view or unique perspective when interpreting and constructing texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1.T.C.1 — Purpose &amp; Audience: Explain how authors of texts use language for a specific purpose and a target audience.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support create texts in teacher-selected modes (e.g., print, digital, auditory, and/or visual) and identify the general purpose (e.g., to tell stories, to provide information, to share opinions, to explain ideas) and target audience in a variety of texts. However, the citations do not cover the standard's other intended skills: identify different modes of communication: print, digital, auditory, and visual. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1.T.C.2 — Authors &amp; Speakers: Investigate the relationships between authors and speakers in texts.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1.T.RA.1 — Research &amp; Inquiry: Build knowledge about the world by asking or generating questions about topics of interest, researching the answers, using multiple sources, and communicating relevant and accurate information about the topic.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fully met</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>This standard is fully met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1.T.RA.2 — Curating Sources &amp; Evidence: Reference parts of texts to address a specific topic or question and explore various sources of information to make connections across a broad range of topics.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support refer to parts of texts when supporting an idea, answer, or opinion. However, the citations do not cover the standard's other intended skills: explore various sources of information, including print, digital, and personal communication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1.T.SS.1 — Organization: Identify and use organizational structures to craft meaning.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support use transition words or phrases, such as once upon a time, next, and last to sequence events and actions. However, the citations do not cover the standard's other intended skills: identify and use various text features (e.g., diagrams, tables of contents) to locate information and make meaning in texts and use text features (e.g., illustrations, page numbers, bold print, headings) to add clarity and meaning to texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1.T.SS.2 — Craft: Identify and use descriptive and engaging language.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fully met</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>This standard is fully met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1.T.T.1 — Narrative Techniques: Identify and use narrative techniques to shape understanding.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support identify a simple plot with a problem and solution, identify techniques used to craft stories, including characters, setting, major events, and dialogue, and describe traits of the main characters and explain how their words and actions support the central message, lesson, or moral of the story. However, the citations do not cover the standard's other intended skills: with adult support, compare and contrast characters and their experiences in stories across diverse cultures and use knowledge of narrative techniques (e.g., characters, settings, events) to create texts that share real or imagined experiences and events with a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1.T.T.2 — Expository Techniques: Identify and use expository techniques to shape understanding.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support identify techniques used to craft expository texts, including main topic and supporting details. However, the citations do not cover the standard's other intended skills: describe the connection between two individuals, events, ideas, or pieces of information in a text and use knowledge of expository techniques to introduce a topic, supply facts about the topic, and provide a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1.T.T.3 — Opinion Techniques: Identify and use opinion techniques to shape understanding.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Beyond scope</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>This standard is beyond the scope of this program module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Texts</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1.T.T.4 — Poetic Techniques: Identify and use poetic techniques to shape understanding.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>This standard is partially met. Citations support use poetic techniques to create poems using simple words and/or phrases that may or may not rhyme. However, the citations do not cover the standard's other intended skills: identify and describe poetic techniques used to craft texts, including rhyme, alliteration, and repeated lines.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>client_format_version</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1.2-client-rollup</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>program_name</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EL Education Curriculum</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>guide_label</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Module 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>judge:output/judge</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>include_statuses</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>full,partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>leaf_standards_with_citations</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>leaf_standards_total</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>135</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>parents_partially_met</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lock Batch-1 pipeline docs and client deliverables after chunk removal.
Drop lesson chunking from the live path, refresh flow diagrams and READMEs, align client correlation parent rollups with the fixed DOCX layout, and regenerate gold-4 result CSVs plus the Module 2 client package.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/veramynd/veramynd_parser/output/reports/GA_ELA_G1_Module2_client_correlation.xlsx
+++ b/veramynd/veramynd_parser/output/reports/GA_ELA_G1_Module2_client_correlation.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -495,7 +495,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -530,7 +530,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -553,7 +553,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -565,7 +565,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -588,7 +588,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -600,7 +600,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -623,7 +623,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -635,7 +635,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -658,7 +658,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -670,7 +670,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -705,7 +705,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -728,7 +728,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -740,7 +740,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -763,7 +763,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -775,7 +775,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -810,7 +810,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -833,7 +833,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -845,7 +845,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -868,7 +868,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -880,7 +880,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -903,7 +903,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -915,7 +915,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -938,7 +938,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -950,7 +950,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -985,7 +985,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1020,7 +1020,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1055,7 +1055,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1090,7 +1090,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1125,7 +1125,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1160,7 +1160,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1195,7 +1195,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1230,7 +1230,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1265,7 +1265,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1300,7 +1300,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1370,7 +1370,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1405,7 +1405,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1463,8 +1463,8 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the select clause is not met — the teacher assigns the text and photos; students never choose their own texts. Per F13, write-without-select is partial, not none.
-Module 2: pp. 44, 99</t>
+          <t>This standard is partially met. The select clause is not met: students never choose their own texts — the teacher assigns the read-aloud ("Elvin, the Boy Who Loved the Sky") and the mystery sky photos.
+Module 2: pp. 48, 102</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1534,23 +1534,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>This standard is partially met. Students also review group norms via the Classroom Discussion Norms anchor chart, partially meeting the develop-norms clause.
-Module 2: pp. 45, 58, 70, 79, 90, 109, 133, 145, 151, 163, 180, 190, 291, 313, 444</t>
+          <t>This standard is partially met. The lesson partially meets 1.P.EICC.1.e. Students also review existing Classroom Discussion Norms ("Direct students' attention to the Classroom Discussion Norms anchor chart and quickly review their jobs as speakers and listeners"), which partially meets the develop-group-norms…
+Module 2: pp. 45, 58, 70, 79, 90, 109, 133, 145, 151, 163, 166, 180, 190, 205, 291, 313, 444</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L7, G1M2U1L9, G1M2U2L10, G1M2U2L8, G1M2U3L11</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L7, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8, G1M2U3L11</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L13, G1M2U2L1</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1606,19 +1610,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, students do not construct/create their own story sharing a real or imagined experience in this lesson — the response sheet records details from the read-aloud text, not an original narrative.
-Module 2: pp. 70, 390</t>
+          <t>This standard is partially met. The interpretation (I) clause is only partially met: students interpret the model poem by identifying high-quality writing features ("What is something you saw or heard in the poem that let you know the poem is high quality?"), but this interpretation focuses on craft quality…
+Module 2: pp. 389</t>
         </is>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>G1M2U1L3, G1M2U3L5</t>
+          <t>G1M2U3L5</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -1642,22 +1646,26 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Module 2: pp. 44, 59, 68, 79, 102, 109, 118, 141, 151, 161, 171, 188, 227, 237, 257, 279, 291, 301, 324, 332, 350, 361, 399, 445, 456, 463</t>
+          <t>Module 2: pp. 45, 59, 70, 79, 83, 102, 109, 118, 125, 141, 151, 161, 171, 180, 188, 205, 227, 237, 257, 279, 291, 301, 307, 324, 332, 350, 361, 366, 380, 399, 404, 414, 424, 445, 456, 463</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>26</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L6</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L5, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U3L3, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1677,22 +1685,26 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Module 2: pp. 44, 59, 70, 78, 89, 103, 109, 141, 161, 171, 180, 188, 213, 291, 311</t>
+          <t>Module 2: pp. 43, 59, 70, 78, 89, 99, 109, 125, 141, 151, 161, 171, 180, 188, 213, 291, 311</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L9</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1712,21 +1724,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is partially met. partial-or-none — The interpretation clause is partially met: students are asked "What is something you saw or heard in the poem that let you know the poem is high quality?" which invites evaluative noticing of the model poem, but the act stays at the observational/noticing…
+Module 2: pp. 389</t>
         </is>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>This standard is beyond the scope of this program module.</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>G1M2U3L5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1747,7 +1760,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1759,7 +1772,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -1782,7 +1795,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1794,7 +1807,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -1817,7 +1830,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1829,7 +1842,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -1852,7 +1865,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1864,7 +1877,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -1887,7 +1900,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1899,7 +1912,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -1922,8 +1935,8 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, there is no activity where students track or revisit their predictions as the reading progresses — the lesson moves through paragraphs with comprehension questions but never returns to confirm or revise the initial prediction.
-Module 2: pp. 44, 99</t>
+          <t>This standard is partially met. The make-predictions clause is partially met: in Opening A, students are asked "Based on the title of the story, what do you think this story will be about?" and they respond with predictions (e.g., "a little boy who likes things in the sky").
+Module 2: pp. 43, 99</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1937,8 +1950,16 @@
           <t>G1M2U1L1, G1M2U1L6</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>input_scope_caveat present on one or more lesson rows</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1958,8 +1979,8 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>This standard is partially met. partial-or-none — In the Mini Language Dive (For ELLs), students infer the meaning of a verse: "What does this verse mean?" (Responses will vary.) and "Now what do you think the verse means?" — a genuine make-inference act about meaning within the text.
-Module 2: pp. 100</t>
+          <t>This standard is partially met. partial-or-full — The make clause is partially met: students are directed to infer why the sun will be at one corner of the page ("With your partner, discuss why you think the sun will be at one corner of the page at the end of the story.
+Module 2: pp. 99</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1973,8 +1994,16 @@
           <t>G1M2U1L6</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>input_scope_caveat present on one or more lesson rows</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1994,7 +2023,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Module 2: pp. 100, 151, 161</t>
+          <t>Module 2: pp. 99, 151, 161</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2029,7 +2058,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2041,7 +2070,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2064,7 +2093,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2076,7 +2105,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2099,18 +2128,18 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Module 2: pp. 44, 58, 66, 91, 100, 134, 144, 188, 213, 289, 311</t>
+          <t>Module 2: pp. 58, 91, 99, 134, 144, 188, 213, 289, 311</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
+          <t>G1M2U1L10, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L8</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2134,22 +2163,26 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Module 2: pp. 290, 312, 323, 381, 409, 420, 428, 436</t>
+          <t>Module 2: pp. 125, 290, 312, 323, 381, 409, 420, 428, 436</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>5</v>
       </c>
       <c r="F49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>G1M2U2L10, G1M2U2L11, G1M2U2L8, G1M2U3L10, G1M2U3L4, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L8, G1M2U3L10, G1M2U3L4, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2204,22 +2237,26 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Module 2: pp. 392, 423, 430, 447</t>
+          <t>Module 2: pp. 375, 391, 423, 430, 432, 447</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>G1M2U3L11, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10, G1M2U3L4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2275,7 +2312,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2287,7 +2324,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2310,19 +2347,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, per F21, the research clause is not met — the teacher-assigned read-aloud, photos, and videos are content delivery, not student-initiated informal research.
-Module 2: pp. 47</t>
+          <t>This standard is partially met. The lesson partially addresses 1.P.ST.1.a. However, these discussions focus on noticing and wondering about content rather than explicitly identifying the key components of context most relevant to interpreting or constructing texts.
+Module 2: pp. 43, 99</t>
         </is>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>G1M2U1L1</t>
+          <t>G1M2U1L1, G1M2U1L6</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
@@ -2346,7 +2383,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2358,7 +2395,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2452,7 +2489,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2464,7 +2501,7 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -2523,7 +2560,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, no activity asks students to analyze or explain how these elements affect the audience or support the text's purpose — the analyze/explain clause is not met.
+          <t>This standard is partially met. However, the lesson does not have students analyze how these elements affect the audience or explain/evaluate how they support the text's purpose; those higher-order clauses are entirely absent.
 Module 2: pp. 70</t>
         </is>
       </c>
@@ -2559,7 +2596,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -2571,7 +2608,7 @@
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -2594,7 +2631,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2606,7 +2643,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -2629,7 +2666,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2641,7 +2678,7 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -2664,7 +2701,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2676,7 +2713,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -2699,23 +2736,27 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>This standard is partially met. Students craft words and phrases for their poem verse using the Adjectives anchor chart and model poem (Work Time A-B), and write a closing to "tell the reader that night is coming to an end." However, the lesson does not explicitly direct students to consider how their…
-Module 2: pp. 390</t>
+          <t>This standard is partially met. [REJECTED: evidence missing or not found in lesson raw text].
+Module 2: pp. 381, 389, 432</t>
         </is>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>G1M2U3L5</t>
+          <t>G1M2U3L10, G1M2U3L4, G1M2U3L5</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2735,7 +2776,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2747,7 +2788,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -2770,7 +2811,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2782,7 +2823,7 @@
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -2805,23 +2846,26 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>This standard is partially met. The explore/interpret side is thin: students answer one question about high-quality features in the model poem (Opening A: "What is something you saw or heard in the poem that let you know the poem is high quality?") but do not substantively analyze how features impact meaning,…
-Module 2: pp. 389</t>
+          <t>Module 2: pp. 217, 389, 432</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>G1M2U3L5</t>
+          <t>G1M2U2L2, G1M2U3L10, G1M2U3L5</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L2, G1M2U3L10</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2841,7 +2885,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -2853,7 +2897,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -2876,7 +2920,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2888,7 +2932,7 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -2911,23 +2955,26 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>This standard is partially met. The consume clause is partially met: students engage with multiple modes — a poem ("Display the 'What We See: The Sun, Moon, and Stars' poem"), photographs ("Display sun photograph 2 and moon photograph 2"), and a video ("As they watch the video, they should look carefully to…
-Module 2: pp. 235, 281, 364, 418</t>
+          <t>Module 2: pp. 235, 281, 364, 375, 389, 394, 418, 432</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>G1M2U2L3, G1M2U2L7, G1M2U3L2, G1M2U3L8</t>
+          <t>G1M2U2L3, G1M2U2L7, G1M2U3L10, G1M2U3L2, G1M2U3L4, G1M2U3L5, G1M2U3L6, G1M2U3L8</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10, G1M2U3L4, G1M2U3L6</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2947,7 +2994,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -2959,7 +3006,7 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -3017,18 +3064,18 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 171, 381, 389, 419, 428, 444</t>
+          <t>Module 2: pp. 45, 171, 381, 389, 419, 428, 436, 444</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F74" t="n">
         <v>3</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L13, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L13, G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -3052,18 +3099,18 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 58, 70, 81, 89, 99, 109, 118, 130, 145, 151, 161, 188, 214, 223, 235, 245, 255, 268, 279, 301, 313, 324, 332, 352, 365, 373, 381, 389, 399, 408, 419, 428, 436, 448, 456, 463</t>
+          <t>Module 2: pp. 47, 58, 81, 89, 99, 109, 118, 130, 145, 151, 161, 188, 214, 223, 235, 245, 255, 268, 279, 301, 313, 324, 332, 352, 365, 373, 381, 399, 408, 419, 428, 436, 448, 456, 463</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F75" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L15, G1M2U1L2, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -3087,22 +3134,26 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Module 2: pp. 45, 70, 81, 92, 103, 109, 117, 141, 161, 171, 180, 188, 223, 246, 259, 268, 291, 301, 313, 332, 352, 364, 373, 379, 389, 408, 421, 430, 438, 448, 457, 463</t>
+          <t>Module 2: pp. 45, 51, 70, 81, 92, 99, 109, 117, 125, 141, 146, 161, 171, 180, 188, 205, 223, 246, 259, 268, 291, 301, 313, 332, 352, 364, 373, 379, 389, 408, 421, 430, 438, 448, 457, 463</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L10, G1M2U2L12, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L12, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L5, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L11, G1M2U1L2, G1M2U1L9, G1M2U2L1</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3122,7 +3173,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -3134,7 +3185,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3157,7 +3208,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -3169,7 +3220,7 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3192,8 +3243,8 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the ask clause is not met — every text-dependent and discussion question is teacher-posed; students only respond.
-Module 2: pp. 47, 70, 102</t>
+          <t>This standard is partially met. The ask clause is not fully met: students are prompted to share "wonders" using the frame "I wonder ___________," and the ELL scaffold models wonder-to-question conversion, but the lesson never scripts a moment where students pose a genuine question to a partner or audience…
+Module 2: pp. 47, 61, 99</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -3207,8 +3258,16 @@
           <t>G1M2U1L1, G1M2U1L3, G1M2U1L6</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Supporting Materials / Read-aloud Guides were not included in the provided Teacher Guide PDF; some comprehension alignments may be understated pending those materials.</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>input_scope_caveat present on one or more lesson rows; missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L3</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3263,7 +3322,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -3275,7 +3334,7 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -3298,7 +3357,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -3310,7 +3369,7 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -3333,7 +3392,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -3345,7 +3404,7 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -3368,7 +3427,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -3380,7 +3439,7 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -3403,7 +3462,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -3415,7 +3474,7 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -3438,7 +3497,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -3450,7 +3509,7 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -3473,7 +3532,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -3485,7 +3544,7 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -3508,7 +3567,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -3520,7 +3579,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -3543,7 +3602,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3555,7 +3614,7 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -3578,7 +3637,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3590,7 +3649,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -3613,7 +3672,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -3625,7 +3684,7 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -3648,7 +3707,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -3660,7 +3719,7 @@
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -3683,7 +3742,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3695,7 +3754,7 @@
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -3718,7 +3777,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -3730,7 +3789,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -3753,7 +3812,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -3765,7 +3824,7 @@
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -3788,7 +3847,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -3800,7 +3859,7 @@
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -3823,7 +3882,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -3835,7 +3894,7 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -3858,7 +3917,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -3870,7 +3929,7 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -3893,7 +3952,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>This standard is partially met. Students independently write verse 3 in complete sentences (Work Time B, p.390): the teacher feedback confirms students turn ideas "into a complete sentence." However, the lesson does not explicitly direct students to use a variety of sentence types or focus on sentence variety…
+          <t>This standard is partially met. However, the lesson never explicitly addresses using a VARIETY of simple sentences or varying sentence TYPES (declarative, interrogative, exclamatory, imperative) — the writing task is structured around a poem model and verse planner, producing sentences but not deliberately…
 Module 2: pp. 390</t>
         </is>
       </c>
@@ -3929,7 +3988,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -3941,7 +4000,7 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -3964,7 +4023,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -3976,7 +4035,7 @@
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -3999,7 +4058,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Module 2: pp. 46, 68, 100, 390</t>
+          <t>Module 2: pp. 45, 70, 99, 389</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -4034,8 +4093,8 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, the deployment occurs primarily in oral partner/small-group discussion settings; the response sheet writing is not explicitly shown to require target vocabulary deployment.
-Module 2: pp. 48, 103, 389</t>
+          <t>This standard is partially met. However, the vocabulary deployment is thin: students use basic content-label words within heavily scaffolded sentence frames rather than demonstrating robust, self-generated use of grade-level vocabulary to communicate meaning.
+Module 2: pp. 39, 99, 389</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -4050,7 +4109,11 @@
         </is>
       </c>
       <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L1</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4070,7 +4133,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -4082,7 +4145,7 @@
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -4105,7 +4168,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -4117,7 +4180,7 @@
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -4140,15 +4203,14 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>This standard is partially met. However, per R3, this act occurs only in supplemental (For ELLs) content, capping the clause at partial.
-Module 2: pp. 100</t>
+          <t>Module 2: pp. 99</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -4176,7 +4238,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -4188,7 +4250,7 @@
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -4211,7 +4273,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -4223,7 +4285,7 @@
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -4246,7 +4308,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -4258,7 +4320,7 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -4281,7 +4343,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Module 2: pp. 100, 390</t>
+          <t>Module 2: pp. 99, 389</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -4352,7 +4414,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4364,7 +4426,7 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -4387,22 +4449,26 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Module 2: pp. 59, 91, 109, 121, 134, 144, 154, 164, 173, 180, 188, 249, 257, 283, 290, 312, 325, 332, 381, 390, 420, 429, 438, 447, 467</t>
+          <t>Module 2: pp. 59, 91, 109, 121, 134, 144, 154, 164, 173, 180, 188, 249, 257, 262, 283, 290, 295, 312, 325, 332, 381, 390, 420, 429, 438, 447, 467</t>
         </is>
       </c>
       <c r="E113" t="n">
         <v>24</v>
       </c>
       <c r="F113" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L4, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U3L10, G1M2U3L11, G1M2U3L13, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L10, G1M2U3L11, G1M2U3L13, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U2L9</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4422,7 +4488,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4434,7 +4500,7 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -4457,7 +4523,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4469,7 +4535,7 @@
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -4492,7 +4558,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4504,7 +4570,7 @@
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -4527,23 +4593,27 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>This standard is partially met. Per F14, a scaffolded (C) frame in which the student performs the act floors at partial, never none. However, the transition phrase is pre-printed (not student-selected) and is a single use, so the standard is only partially met.
-Module 2: pp. 102</t>
+          <t>This standard is partially met. However, within this lesson the student uses only one pre-supplied transition phrase ("At the end") in a scaffolded frame rather than independently selecting and deploying multiple transition words/phrases (e.g., once upon a time, next, last) to sequence events and actions.
+Module 2: pp. 94, 125</t>
         </is>
       </c>
       <c r="E117" t="n">
         <v>0</v>
       </c>
       <c r="F117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>G1M2U1L6</t>
+          <t>G1M2U1L6, G1M2U1L9</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L6, G1M2U1L9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4563,22 +4633,26 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Module 2: pp. 67, 121, 141, 180, 233, 244, 279, 380, 399, 444</t>
+          <t>Module 2: pp. 66, 121, 141, 180, 233, 244, 262, 279, 380, 399, 404, 444</t>
         </is>
       </c>
       <c r="E118" t="n">
         <v>5</v>
       </c>
       <c r="F118" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L14, G1M2U1L3, G1M2U1L8, G1M2U2L3, G1M2U2L4, G1M2U2L7, G1M2U3L11, G1M2U3L4, G1M2U3L6</t>
+          <t>G1M2U1L10, G1M2U1L14, G1M2U1L3, G1M2U1L8, G1M2U2L3, G1M2U2L4, G1M2U2L6, G1M2U2L7, G1M2U3L11, G1M2U3L4, G1M2U3L6, G1M2U3L7</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U3L7</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4598,22 +4672,26 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Module 2: pp. 121, 144, 180, 222, 249, 260, 283, 293, 316, 325, 381, 390, 420, 428, 445</t>
+          <t>Module 2: pp. 121, 144, 180, 222, 249, 260, 262, 283, 293, 295, 316, 325, 381, 389, 420, 428, 432, 445</t>
         </is>
       </c>
       <c r="E119" t="n">
         <v>6</v>
       </c>
       <c r="F119" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L14, G1M2U1L8, G1M2U2L10, G1M2U2L11, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L7, G1M2U2L8, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L10, G1M2U1L14, G1M2U1L8, G1M2U2L10, G1M2U2L11, G1M2U2L2, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U2L6, G1M2U2L9, G1M2U3L10</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4634,7 +4712,7 @@
       <c r="D120" t="inlineStr">
         <is>
           <t>This standard is partially met. The major events clause is only partially met — students discuss what Moon saw and why he changed his mind, but the lesson explicitly defers completing the events section of the Story Elements board to the next lesson, and no question directly asks students to identify the…
-Module 2: pp. 70, 100, 109, 141, 161, 171, 180</t>
+Module 2: pp. 70, 99, 109, 141, 161, 171, 180</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4713,18 +4791,18 @@
       <c r="D122" t="inlineStr">
         <is>
           <t>This standard is partially met. (bored and lonely)") and on the response sheet using a word bank of adjectives (curious, bored, angry, confused) with the frame "I think Moon was _________ because __________." The clause "explain how the characters' actions support the central message, lesson, or moral" is…
-Module 2: pp. 100, 118, 141, 151, 180</t>
+Module 2: pp. 118, 141, 151, 180</t>
         </is>
       </c>
       <c r="E122" t="n">
         <v>0</v>
       </c>
       <c r="F122" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L14, G1M2U1L6, G1M2U1L8</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L14, G1M2U1L8</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -4748,7 +4826,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4760,7 +4838,7 @@
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -4783,7 +4861,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4795,7 +4873,7 @@
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -4854,7 +4932,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4866,7 +4944,7 @@
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -4889,7 +4967,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4901,7 +4979,7 @@
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
@@ -4924,7 +5002,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4936,7 +5014,7 @@
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -4959,7 +5037,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4971,7 +5049,7 @@
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -4994,7 +5072,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -5006,7 +5084,7 @@
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -5029,22 +5107,26 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Module 2: pp. 390, 419, 429, 445</t>
+          <t>Module 2: pp. 380, 390, 419, 429, 432, 445</t>
         </is>
       </c>
       <c r="E131" t="n">
         <v>4</v>
       </c>
       <c r="F131" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>G1M2U3L11, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U3L10, G1M2U3L11, G1M2U3L4, G1M2U3L5, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U3L10</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5064,7 +5146,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Module 2: pp. 48</t>
+          <t>Module 2: pp. 45</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -5134,22 +5216,26 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Module 2: pp. 49, 59, 70, 79, 91, 103, 109, 121, 141, 161, 180, 190, 215, 222, 233, 248, 259, 268, 279, 291, 306, 313, 324, 332, 352, 361, 373, 381, 399, 408, 419, 429, 438, 448, 455, 463</t>
+          <t>Module 2: pp. 45, 59, 70, 79, 91, 102, 109, 121, 125, 141, 146, 161, 180, 190, 215, 222, 233, 248, 259, 268, 279, 291, 306, 313, 324, 332, 352, 361, 373, 381, 399, 408, 419, 429, 438, 448, 455, 463</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F134" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>G1M2U1L1, G1M2U1L10, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
+          <t>G1M2U1L1, G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L3, G1M2U1L4, G1M2U1L5, G1M2U1L6, G1M2U1L7, G1M2U1L8, G1M2U1L9, G1M2U2L1, G1M2U2L10, G1M2U2L11, G1M2U2L12, G1M2U2L2, G1M2U2L3, G1M2U2L4, G1M2U2L5, G1M2U2L6, G1M2U2L7, G1M2U2L8, G1M2U2L9, G1M2U3L1, G1M2U3L10, G1M2U3L11, G1M2U3L12, G1M2U3L13, G1M2U3L2, G1M2U3L3, G1M2U3L4, G1M2U3L6, G1M2U3L7, G1M2U3L8, G1M2U3L9</t>
         </is>
       </c>
       <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L11, G1M2U1L9</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5169,18 +5255,18 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Module 2: pp. 91, 100, 130, 141, 151, 161, 171, 180, 188, 213, 312</t>
+          <t>Module 2: pp. 51, 91, 94, 130, 141, 151, 161, 171, 180, 188, 213, 312</t>
         </is>
       </c>
       <c r="E135" t="n">
         <v>5</v>
       </c>
       <c r="F135" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10</t>
+          <t>G1M2U1L10, G1M2U1L11, G1M2U1L12, G1M2U1L13, G1M2U1L14, G1M2U1L15, G1M2U1L2, G1M2U1L5, G1M2U1L6, G1M2U1L9, G1M2U2L1, G1M2U2L10</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -5190,7 +5276,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>input_scope_caveat present on one or more lesson rows</t>
+          <t>input_scope_caveat present on one or more lesson rows; missing evidence_page lessons (Stage-1 page_start used when available): G1M2U1L2, G1M2U1L6</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5298,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -5224,7 +5310,7 @@
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2.</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -5261,7 +5347,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Roll-up statement — CLIENT FORMAT</t>
+          <t>Roll-up statement — CLIENT FORMAT (target)</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5359,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.F.F.1 — Oral &amp; Silent Reading Fluency: Demonstrate oral and silent reading fluency while reading grade-level texts for understanding, self-correcting as necessary to ensure accuracy and aid comprehension.</t>
+          <t>1.F.F.1 — Oral &amp; Silent Reading Fluency</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5283,7 +5369,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to increase sight word vocabulary using decoding skills by reading grade-appropriate regularly and irregularly spelled words, including high-frequency words, in isolation and context with increasing automaticity, read a wide range of grade-level texts aloud with increasing accuracy, read a wide range of grade-level texts aloud with appropriate prosody (phrasing, expression, juncture/pause, or intonation) to demonstrate understanding, or self-correct while reading text (silently or aloud) to improve comprehension and fluency, rereading as necessary.</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5381,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.F.H.1 — Motor Skills &amp; Letter/Word Formation: Use fine motor skills to form legible letters and words in print.</t>
+          <t>1.F.H.1 — Motor Skills &amp; Letter/Word Formation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5305,7 +5391,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to form all uppercase and lowercase letters and words with accuracy and consistency, form words with accuracy and consistency, or use appropriate spacing between letters, words, or sentences across lines on a page.</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5403,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.F.H.2 — Transcription &amp; Handwriting Fluency: Use working memory to transcribe oral language to written text and maintain meaning while writing letters, words, and sentences quickly and accurately.</t>
+          <t>1.F.H.2 — Transcription &amp; Handwriting Fluency</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5327,7 +5413,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support perform basic transcription skills. However, the citations do not cover the standard's other intended skills: build handwriting fluency by forming accurate letters and words with increasing speed.</t>
+          <t>This standard is partially met. Citations show students perform basic transcription skills. However, none of the cited lessons ask students to build handwriting fluency by forming accurate letters and words with increasing speed.</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5425,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.F.P.1 — Phoneme-Grapheme Correspondences: Identify and produce phoneme-grapheme correspondences.</t>
+          <t>1.F.P.1 — Phoneme-Grapheme Correspondences</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5349,7 +5435,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to identify and produce phoneme-grapheme correspondences for frequently used consonant blends and digraphs or identify and produce both long and short vowel sounds for A, E, I, O, U, including final -e and vowel digraphs.</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5447,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.F.P.2 — Decoding with Phonics: Use grade-level phonics skills to decode words in context and in isolation.</t>
+          <t>1.F.P.2 — Decoding with Phonics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5371,7 +5457,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to decode regularly spelled one-syllable words with a variety of spelling patterns (VC, CV, CVC, CVCe, VCC, CCVC, CVCC, CVVC, CCVCC), including high-frequency words, identify and decode parts of irregularly spelled words, including high-frequency words, decode one-syllable nonsense words with a variety of spelling patterns (VC, CV, CVC, CVCe, VCC, CCVC, CVCC, CVVC, CCVCC), or decode two-syllable words with basic patterns by applying knowledge of basic syllable types.</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5469,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.F.P.3 — Encoding with Phonics: Use grade-level phonics skills to encode words in context and in isolation.</t>
+          <t>1.F.P.3 — Encoding with Phonics</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5393,7 +5479,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to encode regularly spelled one-syllable words with a variety of spelling patterns (VC, CVC, CVCe, VCC, CCVC, CVCC, CCVCC), including high-frequency words, identify and encode irregularly spelled words, including high-frequency words, encode one-syllable nonsense words with a variety of spelling patterns (VC, CVC, CVCe, VCC, CCVC, CVCC, CCVCC), or encode two-syllable words with basic patterns by applying knowledge of basic syllable types.</t>
         </is>
       </c>
     </row>
@@ -5405,7 +5491,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.F.PA.4 — Syllables: Identify and manipulate syllables in spoken words.</t>
+          <t>1.F.PA.4 — Syllables</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5415,7 +5501,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to add, delete, or substitute syllables in spoken words.</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5513,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.F.PA.5 — Onsets &amp; Rimes: Blend and segment onsets and rimes in spoken words.</t>
+          <t>1.F.PA.5 — Onsets &amp; Rimes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5437,7 +5523,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to blend onsets and rimes of spoken one-syllable words with blends, digraphs, or trigraphs in the initial and final positions or segment onsets and rimes of spoken one-syllable words with blends, digraphs, or trigraphs in the initial and final positions.</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5535,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.F.PA.6 — Phonemic Awareness: Identify and manipulate the individual sounds in spoken words.</t>
+          <t>1.F.PA.6 — Phonemic Awareness</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5459,7 +5545,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to isolate and pronounce initial, medial, or final sounds in spoken one-syllable words, including words with digraphs and blends, distinguish between short and long vowel sounds in spoken one-syllable words, blend and segment up to five phonemes, including consonant blends and digraphs, in spoken words, or add, delete, or substitute phonemes in spoken one-syllable words with three or more phonemes.</t>
         </is>
       </c>
     </row>
@@ -5471,7 +5557,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1.L.GC.1 — Grammar, Usage, &amp; Mechanics: Learn and apply conventions of Standard English grammar, usage, and mechanics to aid the comprehension of texts and to communicate clearly in written and spoken language.</t>
+          <t>1.L.GC.1 — Grammar, Usage, &amp; Mechanics</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5481,7 +5567,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to form regular plural nouns by adding -s or -es. (Master), form and use verbs by adding -ing, -ed, or -s. (Master), use action verbs. (Master), use adjectives and adverbs. (Continue), use common and proper nouns. (Continue), form and use the simple verb tenses. (Continue), use determiners (articles, possessive determiners, demonstrative adjectives). (Continue), capitalize proper nouns. (Continue), use periods, exclamation marks, or question marks at the end of sentences. (Continue), form plural nouns by changing -y to -ies. (Introduce), use personal pronouns (subject, object, or possessive). (Introduce), use frequently occurring prepositions. (Introduce), use commas to separate items in a series and to format dates, addresses, salutations, or closings. (Introduce), use apostrophes to form contractions and singular possessive nouns. (Introduce), form and use irregular plural nouns. (Introduce), form and use the past tense of irregular verbs. (Introduce), or use coordinating conjunctions to join words, phrases, or clauses. (Introduce).</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5579,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.L.GC.2 — Syntax: Recognize and compose coherent sentences that express complete thoughts.</t>
+          <t>1.L.GC.2 — Syntax</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5503,7 +5589,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support use a variety of simple sentences (including a variety of sentence types) to develop clarity in written texts. However, the citations do not cover the standard's other intended skills: distinguish between complete and incomplete simple sentences, and identify the sentence type (i.e., declarative, imperative, interrogative, and exclamatory), use singular and plural subjects with matching verbs, and with adult support, use adjectives or adverbs to add details or clarify meaning. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students use a variety of simple sentences (including a variety of sentence types) to develop clarity in written texts. However, none of the cited lessons ask students to distinguish between complete and incomplete simple sentences, and identify the sentence type (i.e., declarative, imperative, interrogative, and exclamatory), use singular and plural subjects with matching verbs, or with adult support, use adjectives or adverbs to add details or clarify meaning. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5601,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1.L.V.1 — General, Academic, &amp; Specialized Vocabulary: Acquire and use general, academic, and specialized vocabulary words and phrases in a variety of settings.</t>
+          <t>1.L.V.1 — General, Academic, &amp; Specialized Vocabulary</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5525,7 +5611,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support acquire and apply general, academic, and specialized vocabulary words and phrases through grade-level texts and content and use grade-level general, academic, and specialized vocabulary words and phrases to communicate in a variety of settings. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students acquire and apply general, academic, and specialized vocabulary words and phrases through grade-level texts and content and use grade-level general, academic, and specialized vocabulary words and phrases to communicate in a variety of settings. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5537,7 +5623,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1.L.V.2 — Word Analysis: Acquire and apply word analysis skills to deconstruct and construct words to make meaning.</t>
+          <t>1.L.V.2 — Word Analysis</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5547,7 +5633,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to identify frequently occurring root words (e.g., look) and inflectional endings used to form and comprehend new words (e.g., looks, looked, looking) or construct words using frequently occurring roots words and inflectional endings.</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5645,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1.L.V.3 — Meaning &amp; Purpose: Make connections between words and phrases and use reference materials to determine or clarify word meanings in a variety of settings and for a variety of purposes.</t>
+          <t>1.L.V.3 — Meaning &amp; Purpose</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5569,7 +5655,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support use knowledge of word relationships and learned vocabulary words and phrases when making word choices in speaking and writing and use context within and beyond a sentence to determine or clarify the meaning of unknown and multiple-meaning words and phrases. However, the citations do not cover the standard's other intended skills: identify the relationship between words and their synonyms and antonyms, distinguish shades of meaning among verbs that describe the same general action (e.g., walk, march, strut, prance), and with teacher support, use a picture dictionary or digital resource to clarify the meaning of unknown words and phrases. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students use context within and beyond a sentence to determine or clarify the meaning of unknown and multiple-meaning words and phrases and use knowledge of word relationships and learned vocabulary words and phrases when making word choices in speaking and writing. However, none of the cited lessons ask students to identify the relationship between words and their synonyms and antonyms, distinguish shades of meaning among verbs that describe the same general action (e.g., walk, march, strut, prance), or with teacher support, use a picture dictionary or digital resource to clarify the meaning of unknown words and phrases.</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5667,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1.P.AC.1 — Reading like a Writer: Interpret texts through the author’s lens by identifying, analyzing, and evaluating craft techniques that are connected to the responses, thoughts, decisions, and questions triggered by the text.</t>
+          <t>1.P.AC.1 — Reading like a Writer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5591,7 +5677,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support identify, apply, and analyze the literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements in texts, explaining or evaluating how specific elements affect the target audience and support the text’s purpose. However, the citations do not cover the standard's other intended skills: identify, apply, and analyze important, interesting, or effective uses of language, explaining or evaluating how specific word choices affect the target audience and support the text’s purpose, explain, analyze, and evaluate how the author’s use of sentence structure and syntax affects the target audience and supports the text’s purpose, and describe, analyze, and evaluate the design and organization of the text, explaining how specific formats, structures, patterns, and features influence the audience, contribute to the text’s accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students identify, apply, and analyze the literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements in texts, explaining or evaluating how specific elements affect the target audience and support the text’s purpose. However, none of the cited lessons ask students to identify, apply, and analyze important, interesting, or effective uses of language, explaining or evaluating how specific word choices affect the target audience and support the text’s purpose, explain, analyze, and evaluate how the author’s use of sentence structure and syntax affects the target audience and supports the text’s purpose, or describe, analyze, and evaluate the design and organization of the text, explaining how specific formats, structures, patterns, and features influence the audience, contribute to the text’s accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5689,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1.P.AC.2 — Writing like a Reader: Construct texts with the audience’s experience in mind, basing decisions about craft techniques on context and purpose.</t>
+          <t>1.P.AC.2 — Writing like a Reader</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5613,7 +5699,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support craft words and phrases in order to influence the responses, thoughts, decisions, and questions of the target audience and achieve a specific purpose. However, the citations do not cover the standard's other intended skills: integrate literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements to appeal to target audiences and achieve specific purposes, make decisions about sentence structure and syntax in order to accommodate and influence the audience and achieve a specific purpose, and organize texts by incorporating specific formats, structures, patterns, and features to influence the audience, facilitate accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students craft words and phrases in order to influence the responses, thoughts, decisions, and questions of the target audience and achieve a specific purpose. However, none of the cited lessons ask students to integrate literary, expository, and opinion (grades K-5) or rhetorical (grades 6-12) elements to appeal to target audiences and achieve specific purposes, make decisions about sentence structure and syntax in order to accommodate and influence the audience and achieve a specific purpose, or organize texts by incorporating specific formats, structures, patterns, and features to influence the audience, facilitate accessibility, and support the text’s purpose. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5625,7 +5711,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1.P.AC.3 — Text Design: Consider the impact of text design on audience and purpose when consuming and producing texts across modes and genres.</t>
+          <t>1.P.AC.3 — Text Design</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5635,7 +5721,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support explore and create texts in various modes and genres, developing and applying knowledge of how specific features impact meaning, tone, style, purpose, and audience and consume and produce multimodal texts, integrating a variety of genres, text features, and craft techniques to influence target audiences and achieve specific purposes. However, the citations do not cover the standard's other intended skills: apply knowledge of how mode and genre impact what kinds of ideas and information are included in texts and apply knowledge of how mode and genre impact how ideas and information are structured and arranged in texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students explore and create texts in various modes and genres, developing and applying knowledge of how specific features impact meaning, tone, style, purpose, and audience and consume and produce multimodal texts, integrating a variety of genres, text features, and craft techniques to influence target audiences and achieve specific purposes. However, none of the cited lessons ask students to apply knowledge of how mode and genre impact what kinds of ideas and information are included in texts or apply knowledge of how mode and genre impact how ideas and information are structured and arranged in texts.</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5733,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1.P.CP.1 — Collaboration: Collaborate with others to accomplish shared goals and projects.</t>
+          <t>1.P.CP.1 — Collaboration</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5657,7 +5743,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support collaborate with others to determine group norms, establish goals and procedures, and facilitate productivity when working on shared projects, contribute to discussions and shared projects by offering ideas, listening to the ideas of others, and providing feedback, and work with others to discuss topics, investigate questions, solve problems, and explore and create texts. However, the citations do not cover the standard's other intended skills: arrive to group discussions and collaborative meetings prepared to be an active participant in the work.</t>
+          <t>This standard is partially met. Citations show students collaborate with others to determine group norms, establish goals and procedures, and facilitate productivity when working on shared projects, contribute to discussions and shared projects by offering ideas, listening to the ideas of others, and providing feedback, and work with others to discuss topics, investigate questions, solve problems, and explore and create texts. However, none of the cited lessons ask students to arrive to group discussions and collaborative meetings prepared to be an active participant in the work.</t>
         </is>
       </c>
     </row>
@@ -5669,7 +5755,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.P.CP.2 — Presentation: Use presentation skills to tailor communication to target audiences for specific purposes.</t>
+          <t>1.P.CP.2 — Presentation</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5679,7 +5765,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support communicate clearly to present ideas, information, and texts, build background knowledge by reciting all or part of significant poems and speeches as appropriate by grade level, and engage in dialogue with audiences by asking and answering questions. However, the citations do not cover the standard's other intended skills: integrate modes and genres most appropriate to purpose and audience and vary tone, pace, and nonverbal gestures as appropriate to purpose and audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students communicate clearly to present ideas, information, and texts, build background knowledge by reciting all or part of significant poems and speeches as appropriate by grade level, and engage in dialogue with audiences by asking and answering questions. However, none of the cited lessons ask students to integrate modes and genres most appropriate to purpose and audience or vary tone, pace, and nonverbal gestures as appropriate to purpose and audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5691,7 +5777,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1.P.EICC.1 — Reader &amp; Writer Identity: Build an identity as a reader and writer, developing a repertoire of resources and tools to continuously expand participation as an active consumer and producer of texts.</t>
+          <t>1.P.EICC.1 — Reader &amp; Writer Identity</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5701,7 +5787,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support discuss or write about personal and academic reading and writing preferences, referring to specific techniques, topics, modes, and genres that resonate most, build a repertoire of comprehension and composition skills, strategies, and techniques, drawing from them as needed to aid the interpretation and construction of texts, select, read, and write texts of personal interest and academic relevance to grade-level texts and topics, participate in a community of readers and writers by developing group norms, discussing texts, sharing individual writing, listening as others share their writing, and offering and responding to feedback, and develop independence and autonomy as a reader and writer. However, the citations do not cover the standard's other intended skills: generate, understand, monitor, and discuss personal and academic reading and writing goals, revising as appropriate. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students discuss or write about personal and academic reading and writing preferences, referring to specific techniques, topics, modes, and genres that resonate most, build a repertoire of comprehension and composition skills, strategies, and techniques, drawing from them as needed to aid the interpretation and construction of texts, select, read, and write texts of personal interest and academic relevance to grade-level texts and topics, participate in a community of readers and writers by developing group norms, discussing texts, sharing individual writing, listening as others share their writing, and offering and responding to feedback, and develop independence and autonomy as a reader and writer. However, none of the cited lessons ask students to generate, understand, monitor, and discuss personal and academic reading and writing goals, revising as appropriate. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5713,7 +5799,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1.P.EICC.2 — Engagement &amp; Intention: Engage in written or spoken dialogue as author and audience for a variety of tasks and purposes, making intentional connections within, between, and beyond texts.</t>
+          <t>1.P.EICC.2 — Engagement &amp; Intention</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5723,7 +5809,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support make use of texts to build knowledge, develop skills, make informed decisions, and share information and ideas, explain and learn concepts and processes by interpreting and constructing texts, and share real or imagined experiences by interpreting and constructing texts that tell or include stories. However, the citations do not cover the standard's other intended skills: interpret and construct texts to aid the analysis and evaluation of texts and ideas and consume and produce texts in order to solve problems or influence decisions. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students make use of texts to build knowledge, develop skills, make informed decisions, and share information and ideas, explain and learn concepts and processes by interpreting and constructing texts, share real or imagined experiences by interpreting and constructing texts that tell or include stories, and interpret and construct texts to aid the analysis and evaluation of texts and ideas. However, none of the cited lessons ask students to consume and produce texts in order to solve problems or influence decisions. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5735,8 +5821,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1.P.EICC.3 — Comprehension Strategies: Engage with a range of complex texts for a variety of tasks and purposes, accessing and using strategies for comprehension before, during, and after reading as part of the meaning-making process.
-Comprehension strategies are tools that students should develop throughout their K-12 education as they work to interpret increasingly complex texts. The effectiveness of these strategies depends largely on the texts themselves, the reasons students engage with them, and the preferences and knowledge bases of individual students. For these reasons, students should receive instruction in a variety of comprehension strategies. Students should learn to select and apply strategies flexibly in order to make sense of the text and accomplish their goals.</t>
+          <t>1.P.EICC.3 — Comprehension Strategies</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5746,7 +5831,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support determine the meanings of unfamiliar words and concepts by applying knowledge of context and of academic vocabulary and word parts, make and track predictions about the events and information likely to come next, and make, track, and support inferences about different levels of meaning within the text. However, the citations do not cover the standard's other intended skills: establish a purpose and set goals for reading, monitor comprehension, and adjust as needed, scan and skim the text, making note of structures and sections that might be most useful, draw from, compare, build, and integrate prior knowledge with the material in the text, addressing inconsistencies or gaps and adding to knowledge repertoires as appropriate, and summarize and visualize sections of the text to maintain understanding. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students determine the meanings of unfamiliar words and concepts by applying knowledge of context and of academic vocabulary and word parts, make and track predictions about the events and information likely to come next, and make, track, and support inferences about different levels of meaning within the text. However, none of the cited lessons ask students to establish a purpose and set goals for reading, monitor comprehension, and adjust as needed, scan and skim the text, making note of structures and sections that might be most useful, draw from, compare, build, and integrate prior knowledge with the material in the text, addressing inconsistencies or gaps and adding to knowledge repertoires as appropriate, or summarize and visualize sections of the text to maintain understanding. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5758,7 +5843,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1.P.EICC.4 — Writing Processes: Compose a range of texts for a variety of purposes and audiences, flexibly engaging in writing processes to plan, draft, evaluate, revise, and edit texts.</t>
+          <t>1.P.EICC.4 — Writing Processes</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5768,7 +5853,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support generate ideas for content by assessing prior knowledge, gathering information from texts, and engaging in discussions with others, link ideas and information to the organization plan, highlighting ideas and information that are most relevant, useful, and impactful, construct an initial draft by integrating ideas and information, evaluate the text’s effectiveness based on self-review or feedback from others, determining whether the text matches the purpose and goals for writing, and make changes to the text based on self-evaluation or external feedback, revising the organization, ideas, information, word choices, and craft techniques in order to increase the text’s effectiveness. However, the citations do not cover the standard's other intended skills: establish a purpose and goals for writing and identify a target audience, plan how to organize the text by selecting modes, genres, and structures that will achieve the purpose and meet the needs of the target audience, and edit the text, ensuring it adheres to the conventions of written language. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students generate ideas for content by assessing prior knowledge, gathering information from texts, and engaging in discussions with others, link ideas and information to the organization plan, highlighting ideas and information that are most relevant, useful, and impactful, construct an initial draft by integrating ideas and information, evaluate the text’s effectiveness based on self-review or feedback from others, determining whether the text matches the purpose and goals for writing, and make changes to the text based on self-evaluation or external feedback, revising the organization, ideas, information, word choices, and craft techniques in order to increase the text’s effectiveness. However, none of the cited lessons ask students to establish a purpose and goals for writing and identify a target audience, plan how to organize the text by selecting modes, genres, and structures that will achieve the purpose and meet the needs of the target audience, or edit the text, ensuring it adheres to the conventions of written language. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5865,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1.P.ST.1 — Context: Develop and apply knowledge of key components of context such as background information, geographic location, cultural influences, time period, and contemporary events when interpreting and constructing texts.</t>
+          <t>1.P.ST.1 — Context</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5790,7 +5875,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support use prior knowledge, formal or informal research, and discussions with others to identify the key components of context that are most relevant and explore how context shapes the author’s decisions and the audience’s responses during the interpretation and construction of texts. However, the citations do not cover the standard's other intended skills: consider how context impacts the purposes of the author and the audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students use prior knowledge, formal or informal research, and discussions with others to identify the key components of context that are most relevant and explore how context shapes the author’s decisions and the audience’s responses during the interpretation and construction of texts. However, none of the cited lessons ask students to consider how context impacts the purposes of the author and the audience. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5802,7 +5887,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1.P.ST.2 — Author, Audience, &amp; Purpose: Interpret and construct texts by developing and applying knowledge of the strategies and techniques authors use to accommodate the target audience and achieve the text’s purpose.</t>
+          <t>1.P.ST.2 — Author, Audience, &amp; Purpose</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5812,7 +5897,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support develop and apply knowledge of author, audience, and context to discern and establish the purpose of texts being interpreted or constructed and to evaluate the extent to which those texts achieve those purposes and draw from knowledge of how authors consider context and audience to determine which information and ideas to highlight, which text design is most accessible, which word choices and language structures are most effective, and which craft techniques are most impactful. However, the citations do not cover the standard's other intended skills: draw from knowledge of author, audience, and context to discern and establish a clear point of view or unique perspective when interpreting and constructing texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students develop and apply knowledge of author, audience, and context to discern and establish the purpose of texts being interpreted or constructed and to evaluate the extent to which those texts achieve those purposes and draw from knowledge of how authors consider context and audience to determine which information and ideas to highlight, which text design is most accessible, which word choices and language structures are most effective, and which craft techniques are most impactful. However, none of the cited lessons ask students to draw from knowledge of author, audience, and context to discern and establish a clear point of view or unique perspective when interpreting and constructing texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5909,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1.T.C.1 — Purpose &amp; Audience: Explain how authors of texts use language for a specific purpose and a target audience.</t>
+          <t>1.T.C.1 — Purpose &amp; Audience</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5834,7 +5919,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support create texts in teacher-selected modes (e.g., print, digital, auditory, and/or visual) and identify the general purpose (e.g., to tell stories, to provide information, to share opinions, to explain ideas) and target audience in a variety of texts. However, the citations do not cover the standard's other intended skills: identify different modes of communication: print, digital, auditory, and visual. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students create texts in teacher-selected modes (e.g., print, digital, auditory, and/or visual) and identify the general purpose (e.g., to tell stories, to provide information, to share opinions, to explain ideas) and target audience in a variety of texts. However, none of the cited lessons ask students to identify different modes of communication: print, digital, auditory, and visual. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5846,7 +5931,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1.T.C.2 — Authors &amp; Speakers: Investigate the relationships between authors and speakers in texts.</t>
+          <t>1.T.C.2 — Authors &amp; Speakers</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5856,7 +5941,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to identify who is speaking or telling the story at various points in a text.</t>
         </is>
       </c>
     </row>
@@ -5868,7 +5953,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1.T.RA.1 — Research &amp; Inquiry: Build knowledge about the world by asking or generating questions about topics of interest, researching the answers, using multiple sources, and communicating relevant and accurate information about the topic.</t>
+          <t>1.T.RA.1 — Research &amp; Inquiry</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5878,7 +5963,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>This standard is fully met.</t>
+          <t>This standard is fully met. Citations show students ask questions about topics of interest for research, work collaboratively or individually to conduct research on a shared or personal topic of interest by gathering and organizing information from provided sources (including print, digital, and personal communication) using graphic organizers or other support aids, and share relevant and accurate information through a variety of different modes.</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5975,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1.T.RA.2 — Curating Sources &amp; Evidence: Reference parts of texts to address a specific topic or question and explore various sources of information to make connections across a broad range of topics.</t>
+          <t>1.T.RA.2 — Curating Sources &amp; Evidence</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5900,7 +5985,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support refer to parts of texts when supporting an idea, answer, or opinion. However, the citations do not cover the standard's other intended skills: explore various sources of information, including print, digital, and personal communication.</t>
+          <t>This standard is partially met. Citations show students refer to parts of texts when supporting an idea, answer, or opinion. However, none of the cited lessons ask students to explore various sources of information, including print, digital, and personal communication.</t>
         </is>
       </c>
     </row>
@@ -5912,7 +5997,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1.T.SS.1 — Organization: Identify and use organizational structures to craft meaning.</t>
+          <t>1.T.SS.1 — Organization</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5922,7 +6007,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support use transition words or phrases, such as once upon a time, next, and last to sequence events and actions. However, the citations do not cover the standard's other intended skills: identify and use various text features (e.g., diagrams, tables of contents) to locate information and make meaning in texts and use text features (e.g., illustrations, page numbers, bold print, headings) to add clarity and meaning to texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students use transition words or phrases, such as once upon a time, next, and last to sequence events and actions. However, none of the cited lessons ask students to identify and use various text features (e.g., diagrams, tables of contents) to locate information and make meaning in texts or use text features (e.g., illustrations, page numbers, bold print, headings) to add clarity and meaning to texts. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5934,7 +6019,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1.T.SS.2 — Craft: Identify and use descriptive and engaging language.</t>
+          <t>1.T.SS.2 — Craft</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5944,7 +6029,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>This standard is fully met.</t>
+          <t>This standard is fully met. Citations show students identify and explain the use of descriptive words in texts and use descriptive words to craft engaging texts.</t>
         </is>
       </c>
     </row>
@@ -5956,7 +6041,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1.T.T.1 — Narrative Techniques: Identify and use narrative techniques to shape understanding.</t>
+          <t>1.T.T.1 — Narrative Techniques</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5966,7 +6051,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support identify a simple plot with a problem and solution, identify techniques used to craft stories, including characters, setting, major events, and dialogue, and describe traits of the main characters and explain how their words and actions support the central message, lesson, or moral of the story. However, the citations do not cover the standard's other intended skills: with adult support, compare and contrast characters and their experiences in stories across diverse cultures and use knowledge of narrative techniques (e.g., characters, settings, events) to create texts that share real or imagined experiences and events with a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students identify a simple plot with a problem and solution, identify techniques used to craft stories, including characters, setting, major events, and dialogue, and describe traits of the main characters and explain how their words and actions support the central message, lesson, or moral of the story. However, none of the cited lessons ask students to with adult support, compare and contrast characters and their experiences in stories across diverse cultures or use knowledge of narrative techniques (e.g., characters, settings, events) to create texts that share real or imagined experiences and events with a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -5978,7 +6063,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1.T.T.2 — Expository Techniques: Identify and use expository techniques to shape understanding.</t>
+          <t>1.T.T.2 — Expository Techniques</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5988,7 +6073,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support identify techniques used to craft expository texts, including main topic and supporting details. However, the citations do not cover the standard's other intended skills: describe the connection between two individuals, events, ideas, or pieces of information in a text and use knowledge of expository techniques to introduce a topic, supply facts about the topic, and provide a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
+          <t>This standard is partially met. Citations show students identify techniques used to craft expository texts, including main topic and supporting details. However, none of the cited lessons ask students to describe the connection between two individuals, events, ideas, or pieces of information in a text or use knowledge of expository techniques to introduce a topic, supply facts about the topic, and provide a sense of closure. Where a covered skill appears only in part, student performance is incomplete relative to the full skill named by the standard.</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6085,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1.T.T.3 — Opinion Techniques: Identify and use opinion techniques to shape understanding.</t>
+          <t>1.T.T.3 — Opinion Techniques</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6010,7 +6095,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>This standard is beyond the scope of this program module.</t>
+          <t>This standard is beyond the scope of Module 2. None of the cited lessons ask students to identify techniques used to craft opinion texts, including the author’s opinion and supporting reasons or use knowledge of opinion techniques to create opinion pieces that introduce the topic, state an opinion about the topic, or provides two or more reasons to support the opinion with linking words and and because.</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6107,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1.T.T.4 — Poetic Techniques: Identify and use poetic techniques to shape understanding.</t>
+          <t>1.T.T.4 — Poetic Techniques</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6032,7 +6117,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>This standard is partially met. Citations support use poetic techniques to create poems using simple words and/or phrases that may or may not rhyme. However, the citations do not cover the standard's other intended skills: identify and describe poetic techniques used to craft texts, including rhyme, alliteration, and repeated lines.</t>
+          <t>This standard is partially met. Citations show students use poetic techniques to create poems using simple words and/or phrases that may or may not rhyme. However, none of the cited lessons ask students to identify and describe poetic techniques used to craft texts, including rhyme, alliteration, and repeated lines.</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6191,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>judge:output/judge</t>
+          <t>master:..\docs\Veramynd_ALL40_corrected_master.xlsx</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6214,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">

</xml_diff>